<commit_message>
Update analytical metrics CSV files with revised values
- Modified delta_analytical_net_metrics.csv to reflect updated net metrics.
- Adjusted delta_analytical_node_metrics.csv with new node metrics, including changes to lambda, mu, and throughput values.
- Revised dflt_analytical_net_metrics.csv to include updated average metrics and node metrics for consistency.
</commit_message>
<xml_diff>
--- a/assets/cs1/sheet/pydasa_cs1_dim_vars.xlsx
+++ b/assets/cs1/sheet/pydasa_cs1_dim_vars.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd4428830306c10d/Documents/GitHub/DASA-Design/PyDASA-Case-Studies/assets/cs1/sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="13_ncr:1_{D95395EB-DBE5-4D0C-A905-FDA3E5BFB6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2222844-FF56-4EDA-8ED4-1924873908CD}"/>
+  <xr:revisionPtr revIDLastSave="397" documentId="13_ncr:1_{D95395EB-DBE5-4D0C-A905-FDA3E5BFB6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A09B0224-985C-43D5-9128-20BCACC79703}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4000" yWindow="3967" windowWidth="7540" windowHeight="6000" xr2:uid="{EABAE1E3-9871-4CDD-80AF-2EA34DC987B5}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" xr2:uid="{EABAE1E3-9871-4CDD-80AF-2EA34DC987B5}"/>
   </bookViews>
   <sheets>
     <sheet name="dflt_relevance_lt@3FDUs" sheetId="1" r:id="rId1"/>
@@ -2654,15 +2654,15 @@
         <v>7</v>
       </c>
       <c r="L7" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M7" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N7" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O7" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -2670,15 +2670,15 @@
       </c>
       <c r="P7" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R7" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>33</v>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="U7" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.5">
@@ -3539,15 +3539,15 @@
         <v>req</v>
       </c>
       <c r="L18" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M18" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
-      </c>
-      <c r="N18" s="4">
+        <v>15</v>
+      </c>
+      <c r="N18" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O18" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -3555,15 +3555,15 @@
       </c>
       <c r="P18" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q18" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R18" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S18" s="1" t="str">
         <f t="shared" si="5"/>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="U18" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.5">
@@ -4459,15 +4459,15 @@
         <v>req</v>
       </c>
       <c r="L29" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M29" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N29" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O29" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -4475,15 +4475,15 @@
       </c>
       <c r="P29" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q29" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R29" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S29" s="1" t="str">
         <f t="shared" si="5"/>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="U29" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.5">
@@ -5379,15 +5379,15 @@
         <v>req</v>
       </c>
       <c r="L40" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M40" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N40" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O40" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -5395,15 +5395,15 @@
       </c>
       <c r="P40" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q40" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R40" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S40" s="1" t="str">
         <f t="shared" si="5"/>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="U40" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.5">
@@ -6219,12 +6219,11 @@
         <v>1</v>
       </c>
       <c r="M50" s="1">
-        <f>Table1[[#This Row],[_min]]+1</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N50" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="O50" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -6236,11 +6235,11 @@
       </c>
       <c r="Q50" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R50" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="S50" s="1" t="str">
         <f t="shared" si="5"/>
@@ -6252,7 +6251,7 @@
       </c>
       <c r="U50" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 2}</v>
+        <v>{'low': 1, 'high': 3}</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.5">
@@ -6300,15 +6299,15 @@
         <v>req</v>
       </c>
       <c r="L51" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M51" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N51" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O51" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -6316,15 +6315,15 @@
       </c>
       <c r="P51" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q51" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R51" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S51" s="1" t="str">
         <f t="shared" si="5"/>
@@ -6336,7 +6335,7 @@
       </c>
       <c r="U51" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.5">
@@ -7221,15 +7220,15 @@
         <v>req</v>
       </c>
       <c r="L62" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M62" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N62" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O62" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -7237,15 +7236,15 @@
       </c>
       <c r="P62" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q62" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R62" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S62" s="1" t="str">
         <f t="shared" si="5"/>
@@ -7257,7 +7256,7 @@
       </c>
       <c r="U62" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.5">
@@ -8061,12 +8060,11 @@
         <v>1</v>
       </c>
       <c r="M72" s="1">
-        <f>Table1[[#This Row],[_min]]+1</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N72" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="O72" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -8078,11 +8076,11 @@
       </c>
       <c r="Q72" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R72" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="S72" s="1" t="str">
         <f t="shared" si="5"/>
@@ -8094,7 +8092,7 @@
       </c>
       <c r="U72" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 2}</v>
+        <v>{'low': 1, 'high': 3}</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.5">
@@ -8142,15 +8140,15 @@
         <v>req</v>
       </c>
       <c r="L73" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M73" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N73" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O73" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -8158,15 +8156,15 @@
       </c>
       <c r="P73" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q73" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R73" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S73" s="1" t="str">
         <f t="shared" si="5"/>
@@ -8178,7 +8176,7 @@
       </c>
       <c r="U73" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.5">
@@ -8981,12 +8979,11 @@
         <v>1</v>
       </c>
       <c r="M83" s="1">
-        <f>Table1[[#This Row],[_min]]+1</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N83" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="O83" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -8998,11 +8995,11 @@
       </c>
       <c r="Q83" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R83" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="S83" s="1" t="str">
         <f t="shared" si="113"/>
@@ -9014,7 +9011,7 @@
       </c>
       <c r="U83" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 2}</v>
+        <v>{'low': 1, 'high': 3}</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.5">
@@ -9062,15 +9059,15 @@
         <v>req</v>
       </c>
       <c r="L84" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M84" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N84" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O84" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -9078,15 +9075,15 @@
       </c>
       <c r="P84" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q84" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R84" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S84" s="1" t="str">
         <f t="shared" si="113"/>
@@ -9098,7 +9095,7 @@
       </c>
       <c r="U84" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.5">
@@ -9982,15 +9979,15 @@
         <v>req</v>
       </c>
       <c r="L95" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M95" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N95" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O95" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -9998,15 +9995,15 @@
       </c>
       <c r="P95" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q95" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R95" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S95" s="1" t="str">
         <f t="shared" si="113"/>
@@ -10018,7 +10015,7 @@
       </c>
       <c r="U95" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.5">
@@ -10902,15 +10899,15 @@
         <v>req</v>
       </c>
       <c r="L106" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M106" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N106" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O106" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -10918,15 +10915,15 @@
       </c>
       <c r="P106" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q106" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R106" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S106" s="1" t="str">
         <f t="shared" si="113"/>
@@ -10938,7 +10935,7 @@
       </c>
       <c r="U106" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.5">
@@ -11822,15 +11819,15 @@
         <v>req</v>
       </c>
       <c r="L117" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M117" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N117" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O117" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -11838,15 +11835,15 @@
       </c>
       <c r="P117" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q117" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R117" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S117" s="1" t="str">
         <f t="shared" si="113"/>
@@ -11858,7 +11855,7 @@
       </c>
       <c r="U117" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.5">
@@ -12742,15 +12739,15 @@
         <v>req</v>
       </c>
       <c r="L128" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M128" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N128" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O128" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -12758,15 +12755,15 @@
       </c>
       <c r="P128" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q128" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R128" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S128" s="1" t="str">
         <f t="shared" si="113"/>
@@ -12778,7 +12775,7 @@
       </c>
       <c r="U128" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.5">
@@ -13662,15 +13659,15 @@
         <v>req</v>
       </c>
       <c r="L139" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M139" s="1">
         <f>Table1[[#This Row],[_min]]+10</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N139" s="1">
         <f>AVERAGE(Table1[[#This Row],[_min]:[_max]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O139" s="1" t="str">
         <f>Table1[[#This Row],[_units]]</f>
@@ -13678,15 +13675,15 @@
       </c>
       <c r="P139" s="1">
         <f>Table1[[#This Row],[_min]]</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q139" s="1">
         <f>Table1[[#This Row],[_max]]</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R139" s="1">
         <f>Table1[[#This Row],[_mean]]</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S139" s="1" t="str">
         <f t="shared" si="113"/>
@@ -13698,7 +13695,7 @@
       </c>
       <c r="U139" s="1" t="str">
         <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 1, 'high': 11}</v>
+        <v>{'low': 5, 'high': 15}</v>
       </c>
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.5">

</xml_diff>